<commit_message>
Se organizan archivos para las solicitudes
</commit_message>
<xml_diff>
--- a/backend/src/assets/templates/SOLICITUDES3.xlsx
+++ b/backend/src/assets/templates/SOLICITUDES3.xlsx
@@ -5,10 +5,10 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/3e335d3f3ef462b1/Documentos/COSAS U/SEMESTRE 9/PRACTICAS/PROYECTO/BACKEND/PRACTICAS-BACK/backend/src/assets/templates/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\camig\OneDrive\Documentos\COSAS U\SEMESTRE 9\PRACTICAS\PROYECTO\BACKEND\PRACTICAS-BACK\backend\src\assets\templates\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="7" documentId="8_{B7D75FE1-1960-4686-93C1-D592DFBC71C8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{275C93DD-7D60-44D2-BA7F-399F4EA7E343}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{009AD4A1-56ED-45E8-BE6F-B0604B6E2AF8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" xr2:uid="{F2F517B1-4DB8-440A-BC86-F71603E3430E}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="11" uniqueCount="11">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="15" uniqueCount="15">
   <si>
     <t>N</t>
   </si>
@@ -63,13 +63,25 @@
     <t>DETALLE NOVEDAD</t>
   </si>
   <si>
-    <t>DIAS A TOMAR</t>
-  </si>
-  <si>
-    <t>FECHA INICIO</t>
-  </si>
-  <si>
-    <t>FECHA FIN</t>
+    <t>JORNADA EMPLEADO</t>
+  </si>
+  <si>
+    <t>JORNADA OTRO SI TEMPORAL</t>
+  </si>
+  <si>
+    <t xml:space="preserve">FECHA INICIO </t>
+  </si>
+  <si>
+    <t xml:space="preserve">FECHA FIN </t>
+  </si>
+  <si>
+    <t>SALARIO ACTUAL</t>
+  </si>
+  <si>
+    <t>SALARIO OTRO SI TEMPORAL</t>
+  </si>
+  <si>
+    <t>CONSECUTIVO FORMS</t>
   </si>
 </sst>
 </file>
@@ -99,7 +111,7 @@
       <family val="2"/>
     </font>
   </fonts>
-  <fills count="5">
+  <fills count="4">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -115,12 +127,6 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FF002060"/>
-        <bgColor rgb="FF000000"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="0"/>
         <bgColor rgb="FF000000"/>
       </patternFill>
     </fill>
@@ -152,7 +158,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -162,12 +168,6 @@
     </xf>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -602,10 +602,18 @@
       <c r="K5" s="3" t="s">
         <v>10</v>
       </c>
-      <c r="L5" s="4"/>
-      <c r="M5" s="4"/>
-      <c r="N5" s="5"/>
-      <c r="O5" s="5"/>
+      <c r="L5" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="M5" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="N5" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="O5" s="2" t="s">
+        <v>14</v>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>